<commit_message>
Updated the excel file for executive testing -AkashPatel
</commit_message>
<xml_diff>
--- a/src/test/resources/Executive_testing.xlsx
+++ b/src/test/resources/Executive_testing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2521759_cognizant_com/Documents/Desktop/synergia-automation/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521717\Downloads\Testing\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{E9051B01-D027-4C12-A80E-2E5A34134AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D50E2927-0111-4B6E-8ADA-4152D693C304}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{407A9907-87B1-4100-AE51-87AA45D9CF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0F6097E9-48B7-41C0-96F7-C4412DEF2E97}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>username</t>
   </si>
@@ -59,9 +59,6 @@
     <t>invalid password</t>
   </si>
   <si>
-    <t>both invalid</t>
-  </si>
-  <si>
     <t>Akash.Patel6@cognizant.com</t>
   </si>
   <si>
@@ -72,6 +69,15 @@
   </si>
   <si>
     <t>HyperKid@123</t>
+  </si>
+  <si>
+    <t>invalid username and password</t>
+  </si>
+  <si>
+    <t>Akash6</t>
+  </si>
+  <si>
+    <t>123@akash</t>
   </si>
 </sst>
 </file>
@@ -135,10 +141,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -463,7 +465,7 @@
   <cols>
     <col min="1" max="1" width="26.08984375" customWidth="1"/>
     <col min="2" max="2" width="13.90625" customWidth="1"/>
-    <col min="3" max="3" width="14.54296875" customWidth="1"/>
+    <col min="3" max="3" width="26.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -479,10 +481,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
@@ -490,10 +492,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -501,10 +503,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -512,13 +514,13 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -527,6 +529,7 @@
     <hyperlink ref="A3" r:id="rId2" xr:uid="{FFF4057F-5534-46A0-83F3-8453D97D797C}"/>
     <hyperlink ref="B2" r:id="rId3" xr:uid="{0CF0710E-1F4A-4834-99C2-82962D11FE19}"/>
     <hyperlink ref="B3" r:id="rId4" xr:uid="{C0CF03E3-C707-4E0E-A51E-824A6AB6C43E}"/>
+    <hyperlink ref="B5" r:id="rId5" xr:uid="{641E0536-4E99-4258-8201-BE07BBD4468E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>